<commit_message>
agrego: click ascendente, click descendente
</commit_message>
<xml_diff>
--- a/lista_eventos_vl550v3.xlsx
+++ b/lista_eventos_vl550v3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bizland365-my.sharepoint.com/personal/simon_vargas_bizland_tech/Documents/val_log_reader/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{8FD7A045-08E4-480B-A9E6-368A4095CDFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A6510954-6D55-4FF0-8296-9A873B0F5575}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="8_{8FD7A045-08E4-480B-A9E6-368A4095CDFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6669A954-1507-4C06-BC64-4DD478A59622}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-48" windowWidth="23256" windowHeight="12456" xr2:uid="{3CD72D0F-0109-4709-BAE3-D4DAF02C6335}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="115">
   <si>
     <t>ID</t>
   </si>
@@ -369,6 +369,18 @@
   </si>
   <si>
     <t>FIN  VALIDACION</t>
+  </si>
+  <si>
+    <t>latitud</t>
+  </si>
+  <si>
+    <t>longitud</t>
+  </si>
+  <si>
+    <t>longitude</t>
+  </si>
+  <si>
+    <t>latitude</t>
   </si>
 </sst>
 </file>
@@ -392,7 +404,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -518,25 +530,56 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thick">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
+      <left/>
+      <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -546,14 +589,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -892,7 +940,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B1D1B55-AF86-45B6-9E5B-2D3BFD69756D}">
-  <dimension ref="A1:D58"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="60.36328125" customWidth="1"/>
@@ -900,7 +948,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
@@ -951,13 +999,13 @@
       <c r="C5" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="11"/>
+      <c r="D5" s="10"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <v>5</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="11" t="s">
         <v>109</v>
       </c>
       <c r="C6" s="3" t="s">
@@ -968,7 +1016,7 @@
       <c r="A7" s="7">
         <v>6</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="11" t="s">
         <v>110</v>
       </c>
       <c r="C7" s="3" t="s">
@@ -1422,115 +1470,155 @@
         <v>101</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" s="7">
         <v>48</v>
       </c>
       <c r="B49" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C49" s="9" t="s">
+      <c r="C49" s="15" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D49" s="17"/>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" s="7">
         <v>49</v>
       </c>
       <c r="B50" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C50" s="9" t="s">
+      <c r="C50" s="15" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D50" s="17"/>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" s="7">
         <v>50</v>
       </c>
       <c r="B51" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="C51" s="9" t="s">
+      <c r="C51" s="15" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D51" s="17"/>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52" s="7">
         <v>51</v>
       </c>
       <c r="B52" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C52" s="9" t="s">
+      <c r="C52" s="15" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D52" s="17"/>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" s="7">
         <v>52</v>
       </c>
       <c r="B53" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="C53" s="8" t="s">
+      <c r="C53" s="15" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A54" s="7">
+      <c r="D53" s="17"/>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A54" s="12">
         <v>53</v>
       </c>
       <c r="B54" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="C54" s="8" t="s">
+      <c r="C54" s="15" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A55" s="7">
+      <c r="D54" s="17"/>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A55" s="12">
         <v>54</v>
       </c>
       <c r="B55" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="C55" s="8" t="s">
+      <c r="C55" s="15" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A56" s="7">
+      <c r="D55" s="17"/>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A56" s="12">
         <v>55</v>
       </c>
       <c r="B56" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="C56" s="8" t="s">
+      <c r="C56" s="15" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A57" s="7">
-        <v>56</v>
+      <c r="D56" s="17"/>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A57" s="12">
+        <v>55</v>
       </c>
       <c r="B57" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="C57" s="8" t="s">
+      <c r="C57" s="15" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A58" s="7">
-        <v>57</v>
+      <c r="D57" s="17"/>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A58" s="12">
+        <v>55</v>
       </c>
       <c r="B58" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="C58" s="8" t="s">
+      <c r="C58" s="15" t="s">
         <v>79</v>
       </c>
+      <c r="D58" s="17"/>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A59" s="13">
+        <v>55</v>
+      </c>
+      <c r="B59" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="C59" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="D59" s="17"/>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A60" s="13">
+        <v>55</v>
+      </c>
+      <c r="B60" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="C60" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="D60" s="17"/>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A61" s="13"/>
+      <c r="B61" s="8"/>
+      <c r="C61" s="15"/>
+      <c r="D61" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>